<commit_message>
Add actual W1 points column to GW1 team sheets
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/VFL_2026_Stage1_W1_Report.xlsx
+++ b/output/VFL_2026_Stage1_W1_Report.xlsx
@@ -64,12 +64,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,9 +96,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,8 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,10 +520,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Actual Pts</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>With IGL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>IGL?</t>
         </is>
@@ -560,9 +572,15 @@
         <v>12.5</v>
       </c>
       <c r="H2" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J2" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>IGL</t>
         </is>
@@ -601,9 +619,15 @@
         <v>11.3</v>
       </c>
       <c r="H3" t="n">
+        <v>11</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="J3" t="n">
         <v>11.3</v>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -638,9 +662,15 @@
         <v>9.5</v>
       </c>
       <c r="H4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="J4" t="n">
         <v>9.5</v>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -675,9 +705,15 @@
         <v>8.6</v>
       </c>
       <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="J5" t="n">
         <v>8.6</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -712,9 +748,15 @@
         <v>10.1</v>
       </c>
       <c r="H6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="J6" t="n">
         <v>10.1</v>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -749,9 +791,15 @@
         <v>8.300000000000001</v>
       </c>
       <c r="H7" t="n">
+        <v>6</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="J7" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -786,9 +834,15 @@
         <v>7.9</v>
       </c>
       <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J8" t="n">
         <v>7.9</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -823,9 +877,15 @@
         <v>7.5</v>
       </c>
       <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J9" t="n">
         <v>7.5</v>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -860,9 +920,15 @@
         <v>12.3</v>
       </c>
       <c r="H10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="J10" t="n">
         <v>12.3</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -897,9 +963,15 @@
         <v>8.199999999999999</v>
       </c>
       <c r="H11" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="J11" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -934,12 +1006,18 @@
         <v>7.4</v>
       </c>
       <c r="H12" t="n">
+        <v>7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="J12" t="n">
         <v>7.4</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -948,6 +1026,9 @@
         <v>100</v>
       </c>
       <c r="H14" t="n">
+        <v>75</v>
+      </c>
+      <c r="J14" t="n">
         <v>116.2</v>
       </c>
     </row>
@@ -962,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -974,6 +1055,8 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1014,10 +1097,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Actual Pts</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>With IGL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>IGL?</t>
         </is>
@@ -1056,9 +1149,15 @@
         <v>7.6</v>
       </c>
       <c r="H2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J2" t="n">
         <v>7.6</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1093,9 +1192,15 @@
         <v>11.4</v>
       </c>
       <c r="H3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>22.9</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>IGL</t>
         </is>
@@ -1134,9 +1239,15 @@
         <v>8</v>
       </c>
       <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1171,9 +1282,15 @@
         <v>8.4</v>
       </c>
       <c r="H5" t="n">
+        <v>9</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J5" t="n">
         <v>8.4</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1208,9 +1325,15 @@
         <v>9.4</v>
       </c>
       <c r="H6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J6" t="n">
         <v>9.4</v>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1245,9 +1368,15 @@
         <v>7.7</v>
       </c>
       <c r="H7" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J7" t="n">
         <v>7.7</v>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1282,9 +1411,15 @@
         <v>7.9</v>
       </c>
       <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J8" t="n">
         <v>7.9</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1319,9 +1454,15 @@
         <v>6.9</v>
       </c>
       <c r="H9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J9" t="n">
         <v>6.9</v>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1356,9 +1497,15 @@
         <v>10.7</v>
       </c>
       <c r="H10" t="n">
+        <v>15</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J10" t="n">
         <v>10.7</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1393,9 +1540,15 @@
         <v>9</v>
       </c>
       <c r="H11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="J11" t="n">
         <v>9</v>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1430,12 +1583,18 @@
         <v>7.4</v>
       </c>
       <c r="H12" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J12" t="n">
         <v>7.4</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -1444,6 +1603,9 @@
         <v>100</v>
       </c>
       <c r="H14" t="n">
+        <v>98</v>
+      </c>
+      <c r="J14" t="n">
         <v>105.9</v>
       </c>
     </row>
@@ -3269,7 +3431,7 @@
       <c r="G39" t="n">
         <v>12.3</v>
       </c>
-      <c r="H39" s="5" t="n">
+      <c r="H39" s="3" t="n">
         <v>-4.3</v>
       </c>
       <c r="I39" t="n">
@@ -3315,7 +3477,7 @@
       <c r="G40" t="n">
         <v>10.4</v>
       </c>
-      <c r="H40" s="5" t="n">
+      <c r="H40" s="3" t="n">
         <v>-2.4</v>
       </c>
       <c r="I40" t="n">
@@ -3729,7 +3891,7 @@
       <c r="G49" t="n">
         <v>12.5</v>
       </c>
-      <c r="H49" s="5" t="n">
+      <c r="H49" s="3" t="n">
         <v>-5.5</v>
       </c>
       <c r="I49" t="n">
@@ -3867,7 +4029,7 @@
       <c r="G52" t="n">
         <v>9.5</v>
       </c>
-      <c r="H52" s="5" t="n">
+      <c r="H52" s="3" t="n">
         <v>-2.5</v>
       </c>
       <c r="I52" t="n">
@@ -4189,7 +4351,7 @@
       <c r="G59" t="n">
         <v>9.1</v>
       </c>
-      <c r="H59" s="5" t="n">
+      <c r="H59" s="3" t="n">
         <v>-3.1</v>
       </c>
       <c r="I59" t="n">
@@ -4235,7 +4397,7 @@
       <c r="G60" t="n">
         <v>8.9</v>
       </c>
-      <c r="H60" s="5" t="n">
+      <c r="H60" s="3" t="n">
         <v>-2.9</v>
       </c>
       <c r="I60" t="n">
@@ -4281,7 +4443,7 @@
       <c r="G61" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="H61" s="5" t="n">
+      <c r="H61" s="3" t="n">
         <v>-2.2</v>
       </c>
       <c r="I61" t="n">
@@ -4327,7 +4489,7 @@
       <c r="G62" t="n">
         <v>10.1</v>
       </c>
-      <c r="H62" s="5" t="n">
+      <c r="H62" s="3" t="n">
         <v>-4.1</v>
       </c>
       <c r="I62" t="n">
@@ -4373,7 +4535,7 @@
       <c r="G63" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="H63" s="5" t="n">
+      <c r="H63" s="3" t="n">
         <v>-2.3</v>
       </c>
       <c r="I63" t="n">
@@ -4603,7 +4765,7 @@
       <c r="G68" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="H68" s="5" t="n">
+      <c r="H68" s="3" t="n">
         <v>-2.3</v>
       </c>
       <c r="I68" t="n">
@@ -4649,7 +4811,7 @@
       <c r="G69" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="H69" s="5" t="n">
+      <c r="H69" s="3" t="n">
         <v>-2.2</v>
       </c>
       <c r="I69" t="n">
@@ -4787,7 +4949,7 @@
       <c r="G72" t="n">
         <v>10.2</v>
       </c>
-      <c r="H72" s="5" t="n">
+      <c r="H72" s="3" t="n">
         <v>-5.2</v>
       </c>
       <c r="I72" t="n">
@@ -4833,7 +4995,7 @@
       <c r="G73" t="n">
         <v>11.4</v>
       </c>
-      <c r="H73" s="5" t="n">
+      <c r="H73" s="3" t="n">
         <v>-6.4</v>
       </c>
       <c r="I73" t="n">
@@ -4879,7 +5041,7 @@
       <c r="G74" t="n">
         <v>7.4</v>
       </c>
-      <c r="H74" s="5" t="n">
+      <c r="H74" s="3" t="n">
         <v>-2.4</v>
       </c>
       <c r="I74" t="n">
@@ -4925,7 +5087,7 @@
       <c r="G75" t="n">
         <v>7</v>
       </c>
-      <c r="H75" s="5" t="n">
+      <c r="H75" s="3" t="n">
         <v>-2</v>
       </c>
       <c r="I75" t="n">
@@ -4971,7 +5133,7 @@
       <c r="G76" t="n">
         <v>8</v>
       </c>
-      <c r="H76" s="5" t="n">
+      <c r="H76" s="3" t="n">
         <v>-3</v>
       </c>
       <c r="I76" t="n">
@@ -5109,7 +5271,7 @@
       <c r="G79" t="n">
         <v>8.6</v>
       </c>
-      <c r="H79" s="5" t="n">
+      <c r="H79" s="3" t="n">
         <v>-3.6</v>
       </c>
       <c r="I79" t="n">
@@ -5201,7 +5363,7 @@
       <c r="G81" t="n">
         <v>8.9</v>
       </c>
-      <c r="H81" s="5" t="n">
+      <c r="H81" s="3" t="n">
         <v>-4.9</v>
       </c>
       <c r="I81" t="n">
@@ -5247,7 +5409,7 @@
       <c r="G82" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="H82" s="5" t="n">
+      <c r="H82" s="3" t="n">
         <v>-4.7</v>
       </c>
       <c r="I82" t="n">
@@ -5293,7 +5455,7 @@
       <c r="G83" t="n">
         <v>6.6</v>
       </c>
-      <c r="H83" s="5" t="n">
+      <c r="H83" s="3" t="n">
         <v>-2.6</v>
       </c>
       <c r="I83" t="n">
@@ -5339,7 +5501,7 @@
       <c r="G84" t="n">
         <v>7.3</v>
       </c>
-      <c r="H84" s="5" t="n">
+      <c r="H84" s="3" t="n">
         <v>-3.3</v>
       </c>
       <c r="I84" t="n">
@@ -5385,7 +5547,7 @@
       <c r="G85" t="n">
         <v>7.1</v>
       </c>
-      <c r="H85" s="5" t="n">
+      <c r="H85" s="3" t="n">
         <v>-3.1</v>
       </c>
       <c r="I85" t="n">
@@ -5431,7 +5593,7 @@
       <c r="G86" t="n">
         <v>9</v>
       </c>
-      <c r="H86" s="5" t="n">
+      <c r="H86" s="3" t="n">
         <v>-5</v>
       </c>
       <c r="I86" t="n">
@@ -5477,7 +5639,7 @@
       <c r="G87" t="n">
         <v>6.1</v>
       </c>
-      <c r="H87" s="5" t="n">
+      <c r="H87" s="3" t="n">
         <v>-2.1</v>
       </c>
       <c r="I87" t="n">
@@ -5707,7 +5869,7 @@
       <c r="G92" t="n">
         <v>10.1</v>
       </c>
-      <c r="H92" s="5" t="n">
+      <c r="H92" s="3" t="n">
         <v>-7.1</v>
       </c>
       <c r="I92" t="n">
@@ -5753,7 +5915,7 @@
       <c r="G93" t="n">
         <v>7.8</v>
       </c>
-      <c r="H93" s="5" t="n">
+      <c r="H93" s="3" t="n">
         <v>-4.8</v>
       </c>
       <c r="I93" t="n">
@@ -5799,7 +5961,7 @@
       <c r="G94" t="n">
         <v>6.1</v>
       </c>
-      <c r="H94" s="5" t="n">
+      <c r="H94" s="3" t="n">
         <v>-3.1</v>
       </c>
       <c r="I94" t="n">
@@ -5845,7 +6007,7 @@
       <c r="G95" t="n">
         <v>7.3</v>
       </c>
-      <c r="H95" s="5" t="n">
+      <c r="H95" s="3" t="n">
         <v>-4.3</v>
       </c>
       <c r="I95" t="n">
@@ -5937,7 +6099,7 @@
       <c r="G97" t="n">
         <v>5.6</v>
       </c>
-      <c r="H97" s="5" t="n">
+      <c r="H97" s="3" t="n">
         <v>-2.6</v>
       </c>
       <c r="I97" t="n">
@@ -5983,7 +6145,7 @@
       <c r="G98" t="n">
         <v>6.4</v>
       </c>
-      <c r="H98" s="5" t="n">
+      <c r="H98" s="3" t="n">
         <v>-3.4</v>
       </c>
       <c r="I98" t="n">
@@ -6029,7 +6191,7 @@
       <c r="G99" t="n">
         <v>6.2</v>
       </c>
-      <c r="H99" s="5" t="n">
+      <c r="H99" s="3" t="n">
         <v>-3.2</v>
       </c>
       <c r="I99" t="n">
@@ -6075,7 +6237,7 @@
       <c r="G100" t="n">
         <v>7.3</v>
       </c>
-      <c r="H100" s="5" t="n">
+      <c r="H100" s="3" t="n">
         <v>-5.3</v>
       </c>
       <c r="I100" t="n">
@@ -6121,7 +6283,7 @@
       <c r="G101" t="n">
         <v>7.5</v>
       </c>
-      <c r="H101" s="5" t="n">
+      <c r="H101" s="3" t="n">
         <v>-5.5</v>
       </c>
       <c r="I101" t="n">
@@ -6167,7 +6329,7 @@
       <c r="G102" t="n">
         <v>4.9</v>
       </c>
-      <c r="H102" s="5" t="n">
+      <c r="H102" s="3" t="n">
         <v>-2.9</v>
       </c>
       <c r="I102" t="n">
@@ -6213,7 +6375,7 @@
       <c r="G103" t="n">
         <v>4.3</v>
       </c>
-      <c r="H103" s="5" t="n">
+      <c r="H103" s="3" t="n">
         <v>-2.3</v>
       </c>
       <c r="I103" t="n">
@@ -6259,7 +6421,7 @@
       <c r="G104" t="n">
         <v>4.5</v>
       </c>
-      <c r="H104" s="5" t="n">
+      <c r="H104" s="3" t="n">
         <v>-2.5</v>
       </c>
       <c r="I104" t="n">
@@ -6305,7 +6467,7 @@
       <c r="G105" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="H105" s="5" t="n">
+      <c r="H105" s="3" t="n">
         <v>-8.300000000000001</v>
       </c>
       <c r="I105" t="n">
@@ -6351,7 +6513,7 @@
       <c r="G106" t="n">
         <v>7.4</v>
       </c>
-      <c r="H106" s="5" t="n">
+      <c r="H106" s="3" t="n">
         <v>-6.4</v>
       </c>
       <c r="I106" t="n">
@@ -6397,7 +6559,7 @@
       <c r="G107" t="n">
         <v>8</v>
       </c>
-      <c r="H107" s="5" t="n">
+      <c r="H107" s="3" t="n">
         <v>-7</v>
       </c>
       <c r="I107" t="n">
@@ -6443,7 +6605,7 @@
       <c r="G108" t="n">
         <v>6.5</v>
       </c>
-      <c r="H108" s="5" t="n">
+      <c r="H108" s="3" t="n">
         <v>-5.5</v>
       </c>
       <c r="I108" t="n">
@@ -6489,7 +6651,7 @@
       <c r="G109" t="n">
         <v>4.2</v>
       </c>
-      <c r="H109" s="5" t="n">
+      <c r="H109" s="3" t="n">
         <v>-3.2</v>
       </c>
       <c r="I109" t="n">
@@ -6535,7 +6697,7 @@
       <c r="G110" t="n">
         <v>7.1</v>
       </c>
-      <c r="H110" s="5" t="n">
+      <c r="H110" s="3" t="n">
         <v>-7.1</v>
       </c>
       <c r="I110" t="n">
@@ -6581,7 +6743,7 @@
       <c r="G111" t="n">
         <v>6.4</v>
       </c>
-      <c r="H111" s="5" t="n">
+      <c r="H111" s="3" t="n">
         <v>-6.4</v>
       </c>
       <c r="I111" t="n">
@@ -6627,7 +6789,7 @@
       <c r="G112" t="n">
         <v>5.7</v>
       </c>
-      <c r="H112" s="5" t="n">
+      <c r="H112" s="3" t="n">
         <v>-5.7</v>
       </c>
       <c r="I112" t="n">
@@ -6673,7 +6835,7 @@
       <c r="G113" t="n">
         <v>6.2</v>
       </c>
-      <c r="H113" s="5" t="n">
+      <c r="H113" s="3" t="n">
         <v>-6.2</v>
       </c>
       <c r="I113" t="n">
@@ -6719,7 +6881,7 @@
       <c r="G114" t="n">
         <v>5.7</v>
       </c>
-      <c r="H114" s="5" t="n">
+      <c r="H114" s="3" t="n">
         <v>-5.7</v>
       </c>
       <c r="I114" t="n">
@@ -6765,7 +6927,7 @@
       <c r="G115" t="n">
         <v>7.1</v>
       </c>
-      <c r="H115" s="5" t="n">
+      <c r="H115" s="3" t="n">
         <v>-8.1</v>
       </c>
       <c r="I115" t="n">
@@ -7211,7 +7373,7 @@
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -7238,7 +7400,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>OUT: Xross</t>
+          <t>OUT: Marteen</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -7282,7 +7444,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>OUT: Marteen</t>
+          <t>OUT: Xross</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -7695,7 +7857,7 @@
       <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -7722,7 +7884,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>OUT: Lovers rock</t>
+          <t>OUT: Krostaly</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -7744,7 +7906,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>OUT: Krostaly</t>
+          <t>OUT: Jemkin</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -7766,7 +7928,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>OUT: Jemkin</t>
+          <t>OUT: Lovers rock</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -8179,7 +8341,7 @@
       <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -8206,7 +8368,7 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>OUT: Loita</t>
+          <t>OUT: Stax</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -8228,7 +8390,7 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>OUT: Primmie</t>
+          <t>OUT: Loita</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
@@ -8250,7 +8412,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>OUT: Stax</t>
+          <t>OUT: Primmie</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -8663,7 +8825,7 @@
       <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -8690,7 +8852,7 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>OUT: seven</t>
+          <t>OUT: Veqaj</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
@@ -8712,7 +8874,7 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>OUT: Veqaj</t>
+          <t>OUT: seven</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -9147,7 +9309,7 @@
       <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -9174,7 +9336,7 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>OUT: Udotan</t>
+          <t>OUT: Killua</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
@@ -9218,7 +9380,7 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>OUT: Killua</t>
+          <t>OUT: Udotan</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
@@ -9631,7 +9793,7 @@
       <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -10073,7 +10235,7 @@
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -10100,7 +10262,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>OUT: PROFEK</t>
+          <t>OUT: Munchkin</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -10122,7 +10284,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>OUT: Munchkin</t>
+          <t>OUT: xeus</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -10144,7 +10306,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>OUT: xeus</t>
+          <t>OUT: PROFEK</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -10557,7 +10719,7 @@
       <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -10584,7 +10746,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>OUT: Yetujey</t>
+          <t>OUT: Kushy</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -10606,7 +10768,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>OUT: Kushy</t>
+          <t>OUT: Lar0k</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -10628,7 +10790,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>OUT: Lar0k</t>
+          <t>OUT: Yetujey</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -11041,7 +11203,7 @@
       <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -11068,7 +11230,7 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>OUT: Jemkin</t>
+          <t>OUT: BeYN</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -11090,7 +11252,7 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>OUT: Udotan</t>
+          <t>OUT: Jemkin</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
@@ -11112,7 +11274,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>OUT: BeYN</t>
+          <t>OUT: Udotan</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -11525,7 +11687,7 @@
       <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -11574,7 +11736,7 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>OUT: Veqaj</t>
+          <t>OUT: Patmen</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -11596,7 +11758,7 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>OUT: Patmen</t>
+          <t>OUT: Veqaj</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
@@ -12009,7 +12171,7 @@
       <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -12058,7 +12220,7 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>OUT: Primmie</t>
+          <t>OUT: Killua</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
@@ -12080,7 +12242,7 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>OUT: Killua</t>
+          <t>OUT: Primmie</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
@@ -12493,7 +12655,7 @@
       <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -12935,7 +13097,7 @@
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -12962,7 +13124,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>OUT: Lar0k</t>
+          <t>OUT: Jemkin</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -13006,7 +13168,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>OUT: Jemkin</t>
+          <t>OUT: Lar0k</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -13419,7 +13581,7 @@
       <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -13446,7 +13608,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>OUT: PROFEK</t>
+          <t>OUT: Kushy</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -13468,7 +13630,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>OUT: Kushy</t>
+          <t>OUT: xeus</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -13490,7 +13652,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>OUT: xeus</t>
+          <t>OUT: PROFEK</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -13903,7 +14065,7 @@
       <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -13930,7 +14092,7 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>OUT: Yetujey</t>
+          <t>OUT: BeYN</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -13974,7 +14136,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>OUT: BeYN</t>
+          <t>OUT: Yetujey</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -14387,7 +14549,7 @@
       <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -14436,7 +14598,7 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>OUT: Rosé</t>
+          <t>OUT: Killua</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -14458,7 +14620,7 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>OUT: Killua</t>
+          <t>OUT: Rosé</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
@@ -14871,7 +15033,7 @@
       <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -14898,7 +15060,7 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>OUT: Derke</t>
+          <t>OUT: Patmen</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
@@ -14942,7 +15104,7 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>OUT: Patmen</t>
+          <t>OUT: Derke</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
@@ -15355,7 +15517,7 @@
       <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>

</xml_diff>